<commit_message>
feat: Aluminium Joinery Configurator, updates, portal view and optimized view
</commit_message>
<xml_diff>
--- a/static/xls/fillings_import.xlsx
+++ b/static/xls/fillings_import.xlsx
@@ -164,6 +164,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__FENETRE_FIXE__1</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -231,6 +236,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -298,6 +308,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -365,6 +380,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__FENETRE_1_VANTAIL_OSCILLO_BATTANT__1</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -432,6 +452,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__FENETRE_2_VANTAUX_OSCILLO_BATTANT__1</t>
+        </is>
+      </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -499,6 +524,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__FENETRE_A_SOUFFLET__1</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -566,6 +596,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__PORTE_FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -633,6 +668,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__PORTE_FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -700,6 +740,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__PORTE_1_VANTAIL_OUVERTURE_INT_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -767,6 +812,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_A_FRAPPE__PORTE_2_VANTAUX_OUVERTURE_INT_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -834,6 +884,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -901,6 +956,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_3_VANTAUX_ALIGNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -968,6 +1028,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_3_VANTAUX_ALTERNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1035,6 +1100,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1102,6 +1172,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1169,6 +1244,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_4_VANTAUX_4_RAILS__1</t>
+        </is>
+      </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1236,6 +1316,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1303,6 +1388,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_3_VANTAUX_ALIGNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1370,6 +1460,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_3_VANTAUX_ALTERNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1437,6 +1532,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1504,6 +1604,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1571,6 +1676,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__FENETRE_2_VANTAUX_2_RAILS_AVEC_COUVRE_JOINT__1</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1638,6 +1748,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_2_VANTAUX_2_RAILS_AVEC_COUVRE_JOINT__1</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1705,6 +1820,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>FILL__MASAI_COULISSANT__PORTE_FENETRE_4_VANTAUX_4_RAILS__1</t>
+        </is>
+      </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1772,6 +1892,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1839,6 +1964,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_3_VANTAUX_ALIGNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1906,6 +2036,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_3_VANTAUX_ALTERNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -1973,6 +2108,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2040,6 +2180,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_4_VANTAUX_4_RAILS__1</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2107,6 +2252,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F31" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2174,6 +2324,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_3_VANTAUX_ALIGNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F32" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2241,6 +2396,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_3_VANTAUX_ALTERNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F33" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2308,6 +2468,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F34" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2375,6 +2540,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F35" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2442,6 +2612,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_4_VANTAUX_4_RAILS__1</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2509,6 +2684,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_2_VANTAUX_2_RAILS_AVEC_COUVRE_JOINT__1</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2576,6 +2756,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__PORTE_FENETRE_2_VANTAUX_2_RAILS_AVEC_COUVRE_JOINT__1</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2643,6 +2828,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>FILL__FURIO_COULISSANT__FENETRE_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2710,6 +2900,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_FIXE__1</t>
+        </is>
+      </c>
       <c r="F40" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2777,6 +2972,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F41" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2844,6 +3044,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2911,6 +3116,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_1_VANTAIL_OSCILLO_BATTANTE__1</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -2978,6 +3188,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_2_VANTAUX_OSCILLO_BATTANTE__1</t>
+        </is>
+      </c>
       <c r="F44" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3045,6 +3260,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_A_SOUFFLET__1</t>
+        </is>
+      </c>
       <c r="F45" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3112,6 +3332,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__PORTE_FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3179,6 +3404,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__FENETRE_OUVERTURE_A_ITALIENNE__1</t>
+        </is>
+      </c>
       <c r="F47" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3246,6 +3476,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>FILL__TOUNDRA_A_FRAPPE__PORTE_FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F48" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3313,6 +3548,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_FIXE__1</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3380,6 +3620,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_SOUFFLET__1</t>
+        </is>
+      </c>
       <c r="F50" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3447,6 +3692,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F51" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3514,6 +3764,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F52" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3581,6 +3836,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__PORTE_FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F53" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3648,6 +3908,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__PORTE_FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F54" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3715,6 +3980,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_1_VANTAIL_OSCILLO_BATTANTE__1</t>
+        </is>
+      </c>
       <c r="F55" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3782,6 +4052,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_2_VANTAUX_OSCILLO_BATTANTE__1</t>
+        </is>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3849,6 +4124,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__FENETRE_FIXE_DORMANT_COUVRE_JOINT__1</t>
+        </is>
+      </c>
       <c r="F57" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3916,6 +4196,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__PORTE_1_VANTAIL_OUVERTURE_INT_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F58" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -3983,6 +4268,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>FILL__FLAMINGO_A_FRAPPE__PORTE_2_VANTAUX_OUVERTURE_INT_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4050,6 +4340,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_200__FENETRE_FIXE__1</t>
+        </is>
+      </c>
       <c r="F60" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4117,6 +4412,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_200__FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F61" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4184,6 +4484,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_200__FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F62" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4251,6 +4556,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_200__FENETRE_A_SOUFFLET__1</t>
+        </is>
+      </c>
       <c r="F63" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4318,6 +4628,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_200__PORTE_FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F64" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4385,6 +4700,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_200__PORTE_FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F65" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4452,6 +4772,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__FENETRE_FIXE__1</t>
+        </is>
+      </c>
       <c r="F66" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4519,6 +4844,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4586,6 +4916,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F68" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4653,6 +4988,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__FENETRE_A_SOUFFLET__1</t>
+        </is>
+      </c>
       <c r="F69" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4720,6 +5060,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_FENETRE_1_VANTAIL_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F70" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4787,6 +5132,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_FENETRE_2_VANTAUX_OUVERTURE_FRANCAISE__1</t>
+        </is>
+      </c>
       <c r="F71" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4854,6 +5204,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_1_VANTAIL_OUVRANT_INT_PERIPHERIQUE_SANS_SEUIL__1</t>
+        </is>
+      </c>
       <c r="F72" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4921,6 +5276,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_2_VANTAUX_OUVRANT_INT_PERIPHERIQUE_SANS_SEUIL__1</t>
+        </is>
+      </c>
       <c r="F73" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -4988,6 +5348,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_1_VANTAIL_OUVRANT_INT_PLINTHE_SANS_SEUIL__1</t>
+        </is>
+      </c>
       <c r="F74" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5055,6 +5420,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_2_VANTAUX_OUVRANT_INT_PLINTHE_SANS_SEUIL__1</t>
+        </is>
+      </c>
       <c r="F75" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5122,6 +5492,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_1_VANTAIL_OUVRANT_INT_PERIPHERIQUE_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F76" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5189,6 +5564,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_2_VANTAUX_OUVRANT_INT_PERIPHERIQUE_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F77" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5256,6 +5636,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_1_VANTAIL_OUVRANT_INT_PLINTHE_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F78" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5323,6 +5708,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_A_FRAPPE_900__PORTE_2_VANTAUX_OUVRANT_INT_PLINTHE_SEUIL_PLAT__1</t>
+        </is>
+      </c>
       <c r="F79" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5390,6 +5780,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_100__COUPES_COULISSANT_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F80" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5457,6 +5852,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_100__COUPES_COULISSANT_3_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5524,6 +5924,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_100__COUPES_COULISSANT_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F82" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5591,6 +5996,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_SV__COUPES_COULISSANT_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F83" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5658,6 +6068,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_SV__COUPES_COULISSANT_3_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F84" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5725,6 +6140,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_SV__COUPES_COULISSANT_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F85" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5792,6 +6212,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_SV__COUPES_COULISSANT_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F86" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5859,6 +6284,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__FENETRE_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F87" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5926,6 +6356,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__FENETRE_3_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -5993,6 +6428,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__FENETRE_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6060,6 +6500,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__FENETRE_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F90" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6127,6 +6572,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__PORTE_FENETRE_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F91" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6194,6 +6644,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__PORTE_FENETRE_3_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F92" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6261,6 +6716,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__PORTE_FENETRE_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F93" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6328,6 +6788,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_300_DV__PORTE_FENETRE_4_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6395,6 +6860,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_400__COUPES_COULISSANT_2_VANTAUX_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6462,6 +6932,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_400__COUPES_COULISSANT_3_VANTAUX_ALTERNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6529,6 +7004,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_400__COUPES_COULISSANT_3_VANTAUX_ALIGNES_2_RAILS__1</t>
+        </is>
+      </c>
       <c r="F97" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6596,6 +7076,11 @@
           <t>Remplissage 1</t>
         </is>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_400__COUPES_COULISSANT_3_VANTAUX_3_RAILS__1</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
           <t>fill_dim</t>
@@ -6661,6 +7146,11 @@
       <c r="D99" t="inlineStr">
         <is>
           <t>Remplissage 1</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>FILL__COMFORT_COULISSANT_400__COUPES_COULISSANT_4_VANTAUX_2_RAILS__1</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">

</xml_diff>